<commit_message>
Marketing tracker: East/Southwest Georgia are no-reply, not declined
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/marketing/campaign-tracker.xlsx
+++ b/docs/marketing/campaign-tracker.xlsx
@@ -3281,12 +3281,12 @@
       <c r="M38" s="19" t="inlineStr"/>
       <c r="N38" s="19" t="inlineStr">
         <is>
-          <t>Declined</t>
+          <t>No reply</t>
         </is>
       </c>
       <c r="O38" s="19" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Second-touch note (week1-followups.md template)</t>
         </is>
       </c>
     </row>
@@ -3350,12 +3350,12 @@
       <c r="M39" s="19" t="inlineStr"/>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>Declined</t>
+          <t>No reply</t>
         </is>
       </c>
       <c r="O39" s="19" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Second-touch note (week1-followups.md template)</t>
         </is>
       </c>
     </row>
@@ -7195,7 +7195,7 @@
       <c r="G7" s="19" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>Fill Fridays from Gmail (sent/replies), the Operator Ledger (witnesslives.com/operator), and RevenueCat.</t>
         </is>
@@ -7422,7 +7422,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="20" t="inlineStr">
         <is>
           <t>Sample numbers removed 2026-09-09 — every row below is real or empty. Web UTM capture is NOT yet built in the app; fill Visits only once it is.</t>
         </is>
@@ -7856,7 +7856,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="20" t="inlineStr">
         <is>
           <t>Sample numbers removed 2026-09-09 — every row below is real or empty. Web UTM capture is NOT yet built in the app; fill Visits only once it is.</t>
         </is>

</xml_diff>